<commit_message>
Capture project attributes (spec level, site type, storeys, height, basement, complexity, access, occupied) into stg.ProjectInformation and DimProject
</commit_message>
<xml_diff>
--- a/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
+++ b/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -676,66 +676,166 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Base Date</t>
+          <t>Spec Level</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2025-06-01</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Currency</t>
+          <t>Site Type</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>GBP</t>
+          <t>Brownfield</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Programme Length In Weeks</t>
+          <t>Nr of Storeys</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>78</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Programme Type</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Traditional</t>
-        </is>
+          <t>Total Height Ground To Roof</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>13.5</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>GIFA</t>
+          <t>Basement Area</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4250</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>Basement Height</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Complexity Rating</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Access Constraints</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Restricted - live campus</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Occupied?</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Base Date</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Programme Length In Weeks</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Programme Type</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Traditional</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>GIFA</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>4250</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>Fictional sample project for ingestion tests and Stage B demo. SUMMARY first metric pair is Costplan; variance = tender − Costplan.</t>
         </is>

</xml_diff>

<commit_message>
Validate SpecLevel/SiteType/ComplexityRating, tighten attribute column types, consolidate site flags onto DimProject
</commit_message>
<xml_diff>
--- a/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
+++ b/sample_data/DEMO_Tender_Comparison_Workbook.xlsx
@@ -743,10 +743,8 @@
           <t>Complexity Rating</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
+      <c r="B28" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29">

</xml_diff>